<commit_message>
TradeSheets: neon-card sales page with embedded live demo, editing rights in sheets
- Sales page rebuilt in the app's design (white page, black turquoise-neon cards)
  with the tracker app embedded as a live demo (build_site.py injects it via srcdoc)
- Workbooks: input cells editable, formula cells locked (no password)
- Email preview image regenerated from the new hero

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SsUek2LVS4AqK9q8U6FWSe
</commit_message>
<xml_diff>
--- a/business/email-assets/trial-pack/1-Job-Profit-Snapshot.xlsx
+++ b/business/email-assets/trial-pack/1-Job-Profit-Snapshot.xlsx
@@ -139,7 +139,7 @@
     <t xml:space="preserve">Verdict</t>
   </si>
   <si>
-    <t xml:space="preserve">TradeSheets free trial pack · Blue text = your inputs · Black = formulas (don't overwrite) · Full custom setup: reply to the email you got this from.</t>
+    <t xml:space="preserve">TradeSheets free trial pack · Blue text = your inputs · Black = locked formulas (Review &gt; Unprotect Sheet to change) · Full custom setup: reply to the email you got this from.</t>
   </si>
 </sst>
 </file>
@@ -311,9 +311,9 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
@@ -323,17 +323,17 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
     </xf>
     <xf numFmtId="166" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="167" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
     </xf>
     <xf numFmtId="167" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
@@ -343,9 +343,9 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="168" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
     </xf>
     <xf numFmtId="168" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
@@ -990,6 +990,7 @@
       </c>
     </row>
   </sheetData>
+  <sheetProtection sheet="true" formatCells="false" formatColumns="false" formatRows="false" sort="false" autoFilter="false"/>
   <conditionalFormatting sqref="B22">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>AND(B22&lt;&gt;"",B22&lt;$B$13)</formula>

</xml_diff>